<commit_message>
📊 RSI Report — 2026-05-21 [auto]
</commit_message>
<xml_diff>
--- a/output/RSI_Screener_2026-05-21.xlsx
+++ b/output/RSI_Screener_2026-05-21.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NSE500" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,57 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00243F60"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +83,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +481,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NSE500  |  RSI Screener  |  Run: 21-May-2026 07:21 IST  |  0 stocks matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TradingView Link</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Current Price (₹)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Daily RSI</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Weekly RSI</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Monthly RSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Monthly RSI &gt; 60</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Weekly RSI &gt; 60</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Daily RSI 40–45</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>